<commit_message>
sanity fixes: SEO quality validation hang/path bugs, breadcrumb matrix mobile/tablet hidden state
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/data/reports/confirmed-bugs-2026-08-11.xlsx
+++ b/tests/data/reports/confirmed-bugs-2026-08-11.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H19"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -842,9 +842,61 @@
         <v>Confirmed via exhaustive source review (Java model, HTL, JS, live dialog JSON) across both the target component and the one plausible false-positive alternative, not inferred from a single check. Once implemented, will also need live NTT API credentials to verify end-to-end.</v>
       </c>
     </row>
+    <row r="18">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="str">
+        <v>(no ticket — found incidentally)</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Homepage (global-atlantic.html)</v>
+      </c>
+      <c r="D18" t="str">
+        <v>aem-quality-validation.spec.ts — "Homepage meta description has appropriate length"</v>
+      </c>
+      <c r="E18" t="str">
+        <v>The live homepage's &lt;meta name="description"&gt; is 162 characters, 2 over the 160-char recommendation Google uses before truncating search-result snippets.</v>
+      </c>
+      <c r="F18" t="str">
+        <v>Live-verified 2026-08-15 against https://author-p101514-e1845752.adobeaemcloud.com/content/global-atlantic.html: description = "Explore annuities, insurance, and retirement solutions from Global Atlantic, designed to help individuals and institutions achieve long-term financial security. " (162 chars incl. trailing space).</v>
+      </c>
+      <c r="G18" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="H18" t="str">
+        <v>Directly measured string length against the live meta tag, not inferred. Very minor (2 chars over) — a one-line copy trim would resolve it.</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="str">
+        <v>(no ticket — found incidentally)</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Homepage Hero (global-atlantic.html)</v>
+      </c>
+      <c r="D19" t="str">
+        <v>aem-quality-validation.spec.ts — "Homepage has exactly one &lt;h1&gt; element"</v>
+      </c>
+      <c r="E19" t="str">
+        <v>The homepage renders two &lt;h1&gt; elements with identical text (cmp-homepage-hero__headline--back and --front) — the --back copy is a decorative duplicate (display:none, likely used for a text-reveal/animation effect) rather than an authoring mistake, so real-world SEO/accessibility impact is low since display:none content is excluded from the accessibility tree and generally not weighted by search engines. Still technically violates the "exactly one &lt;h1&gt;" best practice at the DOM level.</v>
+      </c>
+      <c r="F19" t="str">
+        <v>Live-verified 2026-08-15: both h1.cmp-homepage-hero__headline--back/--front elements confirmed via querySelectorAll, textContent identical, --back computed style is display:none/visibility:hidden/opacity:0 (no aria-hidden, but display:none alone already excludes it from the accessibility tree).</v>
+      </c>
+      <c r="G19" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H19" t="str">
+        <v>Directly reproduced and root-caused (duplicate exists for a hidden animation layer, not authored content duplication) — low real-world impact given display:none.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H19"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>